<commit_message>
feat: add requirements & env.example
</commit_message>
<xml_diff>
--- a/report_create_service_report.xlsx
+++ b/report_create_service_report.xlsx
@@ -599,7 +599,7 @@
     <row r="1" ht="28" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Test Run Summary — create_service_report  |  2026-07-08 09:10</t>
+          <t>Test Run Summary — create_service_report  |  2026-07-08 18:01</t>
         </is>
       </c>
     </row>
@@ -640,14 +640,14 @@
         <v>77</v>
       </c>
       <c r="C4" s="6" t="n">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="D4" s="7" t="n">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="E4" s="5" t="inlineStr">
         <is>
-          <t>67.5%</t>
+          <t>70.1%</t>
         </is>
       </c>
     </row>
@@ -745,10 +745,10 @@
         <v>4</v>
       </c>
       <c r="C11" s="10" t="n">
-        <v>2</v>
-      </c>
-      <c r="D11" s="11" t="n">
-        <v>2</v>
+        <v>4</v>
+      </c>
+      <c r="D11" s="14" t="n">
+        <v>0</v>
       </c>
       <c r="E11" s="14" t="n">
         <v>0</v>
@@ -5008,7 +5008,7 @@
       <c r="K2" s="16" t="inlineStr"/>
       <c r="L2" s="16" t="inlineStr">
         <is>
-          <t>2026-07-08 09:10</t>
+          <t>2026-07-08 18:01</t>
         </is>
       </c>
     </row>
@@ -5068,7 +5068,7 @@
       <c r="K3" s="18" t="inlineStr"/>
       <c r="L3" s="18" t="inlineStr">
         <is>
-          <t>2026-07-08 09:10</t>
+          <t>2026-07-08 18:01</t>
         </is>
       </c>
     </row>
@@ -5128,7 +5128,7 @@
       <c r="K4" s="16" t="inlineStr"/>
       <c r="L4" s="16" t="inlineStr">
         <is>
-          <t>2026-07-08 09:10</t>
+          <t>2026-07-08 18:01</t>
         </is>
       </c>
     </row>
@@ -5188,7 +5188,7 @@
       <c r="K5" s="18" t="inlineStr"/>
       <c r="L5" s="18" t="inlineStr">
         <is>
-          <t>2026-07-08 09:10</t>
+          <t>2026-07-08 18:01</t>
         </is>
       </c>
     </row>
@@ -5248,7 +5248,7 @@
       <c r="K6" s="16" t="inlineStr"/>
       <c r="L6" s="16" t="inlineStr">
         <is>
-          <t>2026-07-08 09:10</t>
+          <t>2026-07-08 18:01</t>
         </is>
       </c>
     </row>
@@ -5308,7 +5308,7 @@
       <c r="K7" s="18" t="inlineStr"/>
       <c r="L7" s="18" t="inlineStr">
         <is>
-          <t>2026-07-08 09:10</t>
+          <t>2026-07-08 18:01</t>
         </is>
       </c>
     </row>
@@ -5368,7 +5368,7 @@
       <c r="K8" s="16" t="inlineStr"/>
       <c r="L8" s="16" t="inlineStr">
         <is>
-          <t>2026-07-08 09:10</t>
+          <t>2026-07-08 18:01</t>
         </is>
       </c>
     </row>
@@ -5428,7 +5428,7 @@
       <c r="K9" s="18" t="inlineStr"/>
       <c r="L9" s="18" t="inlineStr">
         <is>
-          <t>2026-07-08 09:10</t>
+          <t>2026-07-08 18:01</t>
         </is>
       </c>
     </row>
@@ -5480,7 +5480,7 @@
       <c r="K10" s="16" t="inlineStr"/>
       <c r="L10" s="16" t="inlineStr">
         <is>
-          <t>2026-07-08 09:10</t>
+          <t>2026-07-08 18:01</t>
         </is>
       </c>
     </row>
@@ -5532,7 +5532,7 @@
       <c r="K11" s="18" t="inlineStr"/>
       <c r="L11" s="18" t="inlineStr">
         <is>
-          <t>2026-07-08 09:10</t>
+          <t>2026-07-08 18:01</t>
         </is>
       </c>
     </row>
@@ -5567,9 +5567,9 @@
           <t>pass</t>
         </is>
       </c>
-      <c r="G12" s="22" t="inlineStr">
-        <is>
-          <t>FAIL</t>
+      <c r="G12" s="21" t="inlineStr">
+        <is>
+          <t>PASS</t>
         </is>
       </c>
       <c r="H12" s="16" t="inlineStr">
@@ -5579,22 +5579,18 @@
       </c>
       <c r="I12" s="16" t="inlineStr">
         <is>
-          <t xml:space="preserve">  - waiting for locator("[role='option']").first to be visible</t>
-        </is>
-      </c>
-      <c r="J12" s="22" t="inlineStr">
-        <is>
-          <t>✗ FAIL</t>
-        </is>
-      </c>
-      <c r="K12" s="16" t="inlineStr">
-        <is>
-          <t>playwright._impl._errors.TimeoutError: Locator.wait_for: Timeout 5000ms exceeded.</t>
-        </is>
-      </c>
+          <t>auto-populated Select Organization='Acme Corp'</t>
+        </is>
+      </c>
+      <c r="J12" s="21" t="inlineStr">
+        <is>
+          <t>✓ PASS</t>
+        </is>
+      </c>
+      <c r="K12" s="16" t="inlineStr"/>
       <c r="L12" s="16" t="inlineStr">
         <is>
-          <t>2026-07-08 09:10</t>
+          <t>2026-07-08 18:01</t>
         </is>
       </c>
     </row>
@@ -5629,9 +5625,9 @@
           <t>pass</t>
         </is>
       </c>
-      <c r="G13" s="22" t="inlineStr">
-        <is>
-          <t>FAIL</t>
+      <c r="G13" s="21" t="inlineStr">
+        <is>
+          <t>PASS</t>
         </is>
       </c>
       <c r="H13" s="18" t="inlineStr">
@@ -5641,22 +5637,18 @@
       </c>
       <c r="I13" s="18" t="inlineStr">
         <is>
-          <t xml:space="preserve">  - waiting for locator("[role='option']").first to be visible</t>
-        </is>
-      </c>
-      <c r="J13" s="22" t="inlineStr">
-        <is>
-          <t>✗ FAIL</t>
-        </is>
-      </c>
-      <c r="K13" s="18" t="inlineStr">
-        <is>
-          <t>playwright._impl._errors.TimeoutError: Locator.wait_for: Timeout 5000ms exceeded.</t>
-        </is>
-      </c>
+          <t>auto-populated Select Organization='Acme Corp', Select Customer User='Alice Smith - alice.smith@abc.com'</t>
+        </is>
+      </c>
+      <c r="J13" s="21" t="inlineStr">
+        <is>
+          <t>✓ PASS</t>
+        </is>
+      </c>
+      <c r="K13" s="18" t="inlineStr"/>
       <c r="L13" s="18" t="inlineStr">
         <is>
-          <t>2026-07-08 09:10</t>
+          <t>2026-07-08 18:01</t>
         </is>
       </c>
     </row>
@@ -5703,7 +5695,7 @@
       </c>
       <c r="I14" s="16" t="inlineStr">
         <is>
-          <t>auto-populated name='Service Report For Case #0626400003 - 05:41 PM', Select Organization='Beta LLC', Select Customer User='Bob Johnson - shwetaa@example.com'</t>
+          <t>auto-populated name='Service Report For Case #0626400003 - 10:48 AM', Select Organization='Beta LLC', Select Customer User='Bob Johnson - shwetaa@example.com'</t>
         </is>
       </c>
       <c r="J14" s="21" t="inlineStr">
@@ -5714,7 +5706,7 @@
       <c r="K14" s="16" t="inlineStr"/>
       <c r="L14" s="16" t="inlineStr">
         <is>
-          <t>2026-07-08 09:10</t>
+          <t>2026-07-08 18:01</t>
         </is>
       </c>
     </row>
@@ -5761,7 +5753,7 @@
       </c>
       <c r="I15" s="18" t="inlineStr">
         <is>
-          <t>auto-populated name='Service Report For Case #0626400003 - 05:42 PM', Select Organization='Beta LLC', Select Customer User='Bob Johnson - shwetaa@example.com'</t>
+          <t>auto-populated name='Service Report For Case #0626400003 - 10:49 AM', Select Organization='Beta LLC', Select Customer User='Bob Johnson - shwetaa@example.com'</t>
         </is>
       </c>
       <c r="J15" s="21" t="inlineStr">
@@ -5772,7 +5764,7 @@
       <c r="K15" s="18" t="inlineStr"/>
       <c r="L15" s="18" t="inlineStr">
         <is>
-          <t>2026-07-08 09:10</t>
+          <t>2026-07-08 18:01</t>
         </is>
       </c>
     </row>
@@ -5822,7 +5814,7 @@
       <c r="K16" s="16" t="inlineStr"/>
       <c r="L16" s="16" t="inlineStr">
         <is>
-          <t>2026-07-08 09:10</t>
+          <t>2026-07-08 18:01</t>
         </is>
       </c>
     </row>
@@ -5872,7 +5864,7 @@
       <c r="K17" s="18" t="inlineStr"/>
       <c r="L17" s="18" t="inlineStr">
         <is>
-          <t>2026-07-08 09:10</t>
+          <t>2026-07-08 18:01</t>
         </is>
       </c>
     </row>
@@ -5922,7 +5914,7 @@
       <c r="K18" s="16" t="inlineStr"/>
       <c r="L18" s="16" t="inlineStr">
         <is>
-          <t>2026-07-08 09:10</t>
+          <t>2026-07-08 18:01</t>
         </is>
       </c>
     </row>
@@ -5972,7 +5964,7 @@
       <c r="K19" s="18" t="inlineStr"/>
       <c r="L19" s="18" t="inlineStr">
         <is>
-          <t>2026-07-08 09:10</t>
+          <t>2026-07-08 18:01</t>
         </is>
       </c>
     </row>
@@ -6022,7 +6014,7 @@
       <c r="K20" s="16" t="inlineStr"/>
       <c r="L20" s="16" t="inlineStr">
         <is>
-          <t>2026-07-08 09:10</t>
+          <t>2026-07-08 18:01</t>
         </is>
       </c>
     </row>
@@ -6072,7 +6064,7 @@
       <c r="K21" s="18" t="inlineStr"/>
       <c r="L21" s="18" t="inlineStr">
         <is>
-          <t>2026-07-08 09:10</t>
+          <t>2026-07-08 18:01</t>
         </is>
       </c>
     </row>
@@ -6122,7 +6114,7 @@
       <c r="K22" s="16" t="inlineStr"/>
       <c r="L22" s="16" t="inlineStr">
         <is>
-          <t>2026-07-08 09:10</t>
+          <t>2026-07-08 18:01</t>
         </is>
       </c>
     </row>
@@ -6172,7 +6164,7 @@
       <c r="K23" s="18" t="inlineStr"/>
       <c r="L23" s="18" t="inlineStr">
         <is>
-          <t>2026-07-08 09:10</t>
+          <t>2026-07-08 18:01</t>
         </is>
       </c>
     </row>
@@ -6232,7 +6224,7 @@
       <c r="K24" s="16" t="inlineStr"/>
       <c r="L24" s="16" t="inlineStr">
         <is>
-          <t>2026-07-08 09:10</t>
+          <t>2026-07-08 18:01</t>
         </is>
       </c>
     </row>
@@ -6292,7 +6284,7 @@
       <c r="K25" s="18" t="inlineStr"/>
       <c r="L25" s="18" t="inlineStr">
         <is>
-          <t>2026-07-08 09:10</t>
+          <t>2026-07-08 18:01</t>
         </is>
       </c>
     </row>
@@ -6352,7 +6344,7 @@
       <c r="K26" s="16" t="inlineStr"/>
       <c r="L26" s="16" t="inlineStr">
         <is>
-          <t>2026-07-08 09:10</t>
+          <t>2026-07-08 18:01</t>
         </is>
       </c>
     </row>
@@ -6412,7 +6404,7 @@
       <c r="K27" s="18" t="inlineStr"/>
       <c r="L27" s="18" t="inlineStr">
         <is>
-          <t>2026-07-08 09:10</t>
+          <t>2026-07-08 18:01</t>
         </is>
       </c>
     </row>
@@ -6472,7 +6464,7 @@
       <c r="K28" s="16" t="inlineStr"/>
       <c r="L28" s="16" t="inlineStr">
         <is>
-          <t>2026-07-08 09:10</t>
+          <t>2026-07-08 18:01</t>
         </is>
       </c>
     </row>
@@ -6524,7 +6516,7 @@
       <c r="K29" s="18" t="inlineStr"/>
       <c r="L29" s="18" t="inlineStr">
         <is>
-          <t>2026-07-08 09:10</t>
+          <t>2026-07-08 18:01</t>
         </is>
       </c>
     </row>
@@ -6576,7 +6568,7 @@
       <c r="K30" s="16" t="inlineStr"/>
       <c r="L30" s="16" t="inlineStr">
         <is>
-          <t>2026-07-08 09:10</t>
+          <t>2026-07-08 18:01</t>
         </is>
       </c>
     </row>
@@ -6628,7 +6620,7 @@
       <c r="K31" s="18" t="inlineStr"/>
       <c r="L31" s="18" t="inlineStr">
         <is>
-          <t>2026-07-08 09:10</t>
+          <t>2026-07-08 18:01</t>
         </is>
       </c>
     </row>
@@ -6689,7 +6681,7 @@
       <c r="K32" s="16" t="inlineStr"/>
       <c r="L32" s="16" t="inlineStr">
         <is>
-          <t>2026-07-08 09:10</t>
+          <t>2026-07-08 18:01</t>
         </is>
       </c>
     </row>
@@ -6750,7 +6742,7 @@
       <c r="K33" s="18" t="inlineStr"/>
       <c r="L33" s="18" t="inlineStr">
         <is>
-          <t>2026-07-08 09:10</t>
+          <t>2026-07-08 18:01</t>
         </is>
       </c>
     </row>
@@ -6800,7 +6792,7 @@
       <c r="K34" s="16" t="inlineStr"/>
       <c r="L34" s="16" t="inlineStr">
         <is>
-          <t>2026-07-08 09:10</t>
+          <t>2026-07-08 18:01</t>
         </is>
       </c>
     </row>
@@ -6850,7 +6842,7 @@
       <c r="K35" s="18" t="inlineStr"/>
       <c r="L35" s="18" t="inlineStr">
         <is>
-          <t>2026-07-08 09:10</t>
+          <t>2026-07-08 18:01</t>
         </is>
       </c>
     </row>
@@ -6910,7 +6902,7 @@
       <c r="K36" s="16" t="inlineStr"/>
       <c r="L36" s="16" t="inlineStr">
         <is>
-          <t>2026-07-08 09:10</t>
+          <t>2026-07-08 18:01</t>
         </is>
       </c>
     </row>
@@ -6962,7 +6954,7 @@
       <c r="K37" s="18" t="inlineStr"/>
       <c r="L37" s="18" t="inlineStr">
         <is>
-          <t>2026-07-08 09:10</t>
+          <t>2026-07-08 18:01</t>
         </is>
       </c>
     </row>
@@ -7023,7 +7015,7 @@
       <c r="K38" s="16" t="inlineStr"/>
       <c r="L38" s="16" t="inlineStr">
         <is>
-          <t>2026-07-08 09:10</t>
+          <t>2026-07-08 18:01</t>
         </is>
       </c>
     </row>
@@ -7083,7 +7075,7 @@
       <c r="K39" s="18" t="inlineStr"/>
       <c r="L39" s="18" t="inlineStr">
         <is>
-          <t>2026-07-08 09:10</t>
+          <t>2026-07-08 18:01</t>
         </is>
       </c>
     </row>
@@ -7133,7 +7125,7 @@
       <c r="K40" s="16" t="inlineStr"/>
       <c r="L40" s="16" t="inlineStr">
         <is>
-          <t>2026-07-08 09:10</t>
+          <t>2026-07-08 18:01</t>
         </is>
       </c>
     </row>
@@ -7182,7 +7174,7 @@
       </c>
       <c r="I41" s="18" t="inlineStr">
         <is>
-          <t>No in-progress service reports found for this case</t>
+          <t>The report has been created successfully</t>
         </is>
       </c>
       <c r="J41" s="21" t="inlineStr">
@@ -7193,7 +7185,7 @@
       <c r="K41" s="18" t="inlineStr"/>
       <c r="L41" s="18" t="inlineStr">
         <is>
-          <t>2026-07-08 09:10</t>
+          <t>2026-07-08 18:01</t>
         </is>
       </c>
     </row>
@@ -7252,7 +7244,7 @@
       <c r="K42" s="16" t="inlineStr"/>
       <c r="L42" s="16" t="inlineStr">
         <is>
-          <t>2026-07-08 09:10</t>
+          <t>2026-07-08 18:01</t>
         </is>
       </c>
     </row>
@@ -7312,7 +7304,7 @@
       <c r="K43" s="18" t="inlineStr"/>
       <c r="L43" s="18" t="inlineStr">
         <is>
-          <t>2026-07-08 09:10</t>
+          <t>2026-07-08 18:01</t>
         </is>
       </c>
     </row>
@@ -7372,7 +7364,7 @@
       </c>
       <c r="I44" s="16" t="inlineStr">
         <is>
-          <t>Unable to create Appointment. Staff not available during requested time | Staff not available during requested time</t>
+          <t>The Appointment has been created successfully</t>
         </is>
       </c>
       <c r="J44" s="21" t="inlineStr">
@@ -7383,7 +7375,7 @@
       <c r="K44" s="16" t="inlineStr"/>
       <c r="L44" s="16" t="inlineStr">
         <is>
-          <t>2026-07-08 09:10</t>
+          <t>2026-07-08 18:01</t>
         </is>
       </c>
     </row>
@@ -7442,7 +7434,7 @@
       <c r="K45" s="18" t="inlineStr"/>
       <c r="L45" s="18" t="inlineStr">
         <is>
-          <t>2026-07-08 09:10</t>
+          <t>2026-07-08 18:01</t>
         </is>
       </c>
     </row>
@@ -7513,7 +7505,7 @@
       <c r="K46" s="16" t="inlineStr"/>
       <c r="L46" s="16" t="inlineStr">
         <is>
-          <t>2026-07-08 09:10</t>
+          <t>2026-07-08 18:01</t>
         </is>
       </c>
     </row>
@@ -7583,7 +7575,7 @@
       <c r="K47" s="18" t="inlineStr"/>
       <c r="L47" s="18" t="inlineStr">
         <is>
-          <t>2026-07-08 09:10</t>
+          <t>2026-07-08 18:01</t>
         </is>
       </c>
     </row>
@@ -7654,7 +7646,7 @@
       <c r="K48" s="16" t="inlineStr"/>
       <c r="L48" s="16" t="inlineStr">
         <is>
-          <t>2026-07-08 09:10</t>
+          <t>2026-07-08 18:01</t>
         </is>
       </c>
     </row>
@@ -7715,7 +7707,7 @@
       <c r="K49" s="18" t="inlineStr"/>
       <c r="L49" s="18" t="inlineStr">
         <is>
-          <t>2026-07-08 09:10</t>
+          <t>2026-07-08 18:01</t>
         </is>
       </c>
     </row>
@@ -7776,7 +7768,7 @@
       <c r="K50" s="16" t="inlineStr"/>
       <c r="L50" s="16" t="inlineStr">
         <is>
-          <t>2026-07-08 09:10</t>
+          <t>2026-07-08 18:01</t>
         </is>
       </c>
     </row>
@@ -7837,7 +7829,7 @@
       <c r="K51" s="18" t="inlineStr"/>
       <c r="L51" s="18" t="inlineStr">
         <is>
-          <t>2026-07-08 09:10</t>
+          <t>2026-07-08 18:01</t>
         </is>
       </c>
     </row>
@@ -7887,7 +7879,7 @@
       <c r="K52" s="16" t="inlineStr"/>
       <c r="L52" s="16" t="inlineStr">
         <is>
-          <t>2026-07-08 09:10</t>
+          <t>2026-07-08 18:01</t>
         </is>
       </c>
     </row>
@@ -7948,7 +7940,7 @@
       <c r="K53" s="18" t="inlineStr"/>
       <c r="L53" s="18" t="inlineStr">
         <is>
-          <t>2026-07-08 09:10</t>
+          <t>2026-07-08 18:01</t>
         </is>
       </c>
     </row>
@@ -8000,7 +7992,7 @@
       <c r="K54" s="16" t="inlineStr"/>
       <c r="L54" s="16" t="inlineStr">
         <is>
-          <t>2026-07-08 09:10</t>
+          <t>2026-07-08 18:01</t>
         </is>
       </c>
     </row>
@@ -8060,7 +8052,7 @@
       <c r="K55" s="18" t="inlineStr"/>
       <c r="L55" s="18" t="inlineStr">
         <is>
-          <t>2026-07-08 09:10</t>
+          <t>2026-07-08 18:01</t>
         </is>
       </c>
     </row>
@@ -8127,7 +8119,7 @@
       </c>
       <c r="L56" s="16" t="inlineStr">
         <is>
-          <t>2026-07-08 09:10</t>
+          <t>2026-07-08 18:01</t>
         </is>
       </c>
     </row>
@@ -8194,7 +8186,7 @@
       </c>
       <c r="L57" s="18" t="inlineStr">
         <is>
-          <t>2026-07-08 09:10</t>
+          <t>2026-07-08 18:01</t>
         </is>
       </c>
     </row>
@@ -8261,7 +8253,7 @@
       </c>
       <c r="L58" s="16" t="inlineStr">
         <is>
-          <t>2026-07-08 09:10</t>
+          <t>2026-07-08 18:01</t>
         </is>
       </c>
     </row>
@@ -8328,7 +8320,7 @@
       </c>
       <c r="L59" s="18" t="inlineStr">
         <is>
-          <t>2026-07-08 09:10</t>
+          <t>2026-07-08 18:01</t>
         </is>
       </c>
     </row>
@@ -8388,7 +8380,7 @@
       <c r="K60" s="16" t="inlineStr"/>
       <c r="L60" s="16" t="inlineStr">
         <is>
-          <t>2026-07-08 09:10</t>
+          <t>2026-07-08 18:01</t>
         </is>
       </c>
     </row>
@@ -8436,7 +8428,7 @@
       </c>
       <c r="I61" s="18" t="inlineStr">
         <is>
-          <t>The report has been created successfully</t>
+          <t>The report has been created successfully | The report has been created successfully</t>
         </is>
       </c>
       <c r="J61" s="21" t="inlineStr">
@@ -8447,7 +8439,7 @@
       <c r="K61" s="18" t="inlineStr"/>
       <c r="L61" s="18" t="inlineStr">
         <is>
-          <t>2026-07-08 09:10</t>
+          <t>2026-07-08 18:01</t>
         </is>
       </c>
     </row>
@@ -8506,7 +8498,7 @@
       <c r="K62" s="16" t="inlineStr"/>
       <c r="L62" s="16" t="inlineStr">
         <is>
-          <t>2026-07-08 09:10</t>
+          <t>2026-07-08 18:01</t>
         </is>
       </c>
     </row>
@@ -8552,11 +8544,7 @@
           <t>Service Report is created with all required and pre-populated fields for the selected ticket.</t>
         </is>
       </c>
-      <c r="I63" s="18" t="inlineStr">
-        <is>
-          <t>The report has been created successfully</t>
-        </is>
-      </c>
+      <c r="I63" s="18" t="inlineStr"/>
       <c r="J63" s="21" t="inlineStr">
         <is>
           <t>✓ PASS</t>
@@ -8565,7 +8553,7 @@
       <c r="K63" s="18" t="inlineStr"/>
       <c r="L63" s="18" t="inlineStr">
         <is>
-          <t>2026-07-08 09:10</t>
+          <t>2026-07-08 18:01</t>
         </is>
       </c>
     </row>
@@ -8613,7 +8601,7 @@
       </c>
       <c r="I64" s="16" t="inlineStr">
         <is>
-          <t>The report has been created successfully</t>
+          <t>The report has been created successfully | The report has been created successfully</t>
         </is>
       </c>
       <c r="J64" s="21" t="inlineStr">
@@ -8624,7 +8612,7 @@
       <c r="K64" s="16" t="inlineStr"/>
       <c r="L64" s="16" t="inlineStr">
         <is>
-          <t>2026-07-08 09:10</t>
+          <t>2026-07-08 18:01</t>
         </is>
       </c>
     </row>
@@ -8672,7 +8660,7 @@
       </c>
       <c r="I65" s="18" t="inlineStr">
         <is>
-          <t>The report has been created successfully</t>
+          <t>No in-progress service reports found for this case | The report has been created successfully</t>
         </is>
       </c>
       <c r="J65" s="21" t="inlineStr">
@@ -8683,7 +8671,7 @@
       <c r="K65" s="18" t="inlineStr"/>
       <c r="L65" s="18" t="inlineStr">
         <is>
-          <t>2026-07-08 09:10</t>
+          <t>2026-07-08 18:01</t>
         </is>
       </c>
     </row>
@@ -8754,7 +8742,7 @@
       <c r="K66" s="16" t="inlineStr"/>
       <c r="L66" s="16" t="inlineStr">
         <is>
-          <t>2026-07-08 09:10</t>
+          <t>2026-07-08 18:01</t>
         </is>
       </c>
     </row>
@@ -8823,7 +8811,7 @@
       <c r="K67" s="18" t="inlineStr"/>
       <c r="L67" s="18" t="inlineStr">
         <is>
-          <t>2026-07-08 09:10</t>
+          <t>2026-07-08 18:01</t>
         </is>
       </c>
     </row>
@@ -8901,7 +8889,7 @@
       </c>
       <c r="L68" s="16" t="inlineStr">
         <is>
-          <t>2026-07-08 09:10</t>
+          <t>2026-07-08 18:01</t>
         </is>
       </c>
     </row>
@@ -8979,7 +8967,7 @@
       </c>
       <c r="L69" s="18" t="inlineStr">
         <is>
-          <t>2026-07-08 09:10</t>
+          <t>2026-07-08 18:01</t>
         </is>
       </c>
     </row>
@@ -9056,7 +9044,7 @@
       </c>
       <c r="L70" s="16" t="inlineStr">
         <is>
-          <t>2026-07-08 09:10</t>
+          <t>2026-07-08 18:01</t>
         </is>
       </c>
     </row>
@@ -9106,7 +9094,7 @@
       <c r="K71" s="18" t="inlineStr"/>
       <c r="L71" s="18" t="inlineStr">
         <is>
-          <t>2026-07-08 09:10</t>
+          <t>2026-07-08 18:01</t>
         </is>
       </c>
     </row>
@@ -9160,7 +9148,7 @@
       <c r="K72" s="16" t="inlineStr"/>
       <c r="L72" s="16" t="inlineStr">
         <is>
-          <t>2026-07-08 09:10</t>
+          <t>2026-07-08 18:01</t>
         </is>
       </c>
     </row>
@@ -9214,7 +9202,7 @@
       <c r="K73" s="18" t="inlineStr"/>
       <c r="L73" s="18" t="inlineStr">
         <is>
-          <t>2026-07-08 09:10</t>
+          <t>2026-07-08 18:01</t>
         </is>
       </c>
     </row>
@@ -9264,7 +9252,7 @@
       <c r="K74" s="16" t="inlineStr"/>
       <c r="L74" s="16" t="inlineStr">
         <is>
-          <t>2026-07-08 09:10</t>
+          <t>2026-07-08 18:01</t>
         </is>
       </c>
     </row>
@@ -9322,7 +9310,7 @@
       <c r="K75" s="18" t="inlineStr"/>
       <c r="L75" s="18" t="inlineStr">
         <is>
-          <t>2026-07-08 09:10</t>
+          <t>2026-07-08 18:01</t>
         </is>
       </c>
     </row>
@@ -9380,7 +9368,7 @@
       <c r="K76" s="16" t="inlineStr"/>
       <c r="L76" s="16" t="inlineStr">
         <is>
-          <t>2026-07-08 09:10</t>
+          <t>2026-07-08 18:01</t>
         </is>
       </c>
     </row>
@@ -9438,7 +9426,7 @@
       <c r="K77" s="18" t="inlineStr"/>
       <c r="L77" s="18" t="inlineStr">
         <is>
-          <t>2026-07-08 09:10</t>
+          <t>2026-07-08 18:01</t>
         </is>
       </c>
     </row>
@@ -9503,7 +9491,7 @@
       </c>
       <c r="L78" s="16" t="inlineStr">
         <is>
-          <t>2026-07-08 09:10</t>
+          <t>2026-07-08 18:01</t>
         </is>
       </c>
     </row>

</xml_diff>